<commit_message>
Updated Aurum Daily Percentages workbook
</commit_message>
<xml_diff>
--- a/assets/Aurum Daily Percentages.xlsx
+++ b/assets/Aurum Daily Percentages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4b660e05f479584a/Documents/Aurum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{35D953AC-DC9B-473D-9159-C2034EEE3E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05CDDC2E-B7D8-4FB2-8DFD-79F9E8A426D5}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="8_{35D953AC-DC9B-473D-9159-C2034EEE3E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{901AABD5-0C00-44B1-9E2C-525AC41C9183}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{FC9DB034-314E-4971-BA3F-7D1E305EC0F5}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="23">
   <si>
     <t>March</t>
   </si>
@@ -107,12 +107,15 @@
   <si>
     <t xml:space="preserve">Dec 2026 </t>
   </si>
+  <si>
+    <t>Profits shifted to Neyro Bot</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,8 +164,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -193,6 +203,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -215,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -293,6 +309,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -631,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8B698C8-EA1E-4653-AD30-D34FDA43EED7}">
-  <dimension ref="A1:T35"/>
+  <dimension ref="A1:T37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1660,7 +1679,7 @@
         <v>29</v>
       </c>
       <c r="H30" s="13">
-        <v>0.32</v>
+        <v>0.57999999999999996</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
@@ -1687,6 +1706,9 @@
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
+      <c r="H31" s="13">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="9">
@@ -1732,7 +1754,7 @@
       </c>
       <c r="H33" s="15">
         <f>SUM(H2:H31)/100</f>
-        <v>0.16750000000000001</v>
+        <v>0.17509999999999998</v>
       </c>
       <c r="I33" s="14" t="s">
         <v>10</v>
@@ -1782,7 +1804,10 @@
       <c r="G34" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="H34" s="17"/>
+      <c r="H34" s="17">
+        <f>H35-F35</f>
+        <v>216.82000000000016</v>
+      </c>
       <c r="I34" s="16" t="s">
         <v>11</v>
       </c>
@@ -1830,7 +1855,9 @@
       <c r="G35" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H35" s="19"/>
+      <c r="H35" s="19">
+        <v>2712.48</v>
+      </c>
       <c r="I35" s="18" t="s">
         <v>12</v>
       </c>
@@ -1856,7 +1883,20 @@
       </c>
       <c r="T35" s="19"/>
     </row>
+    <row r="36" spans="1:20" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G36" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="H36" s="27"/>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="G36:H36"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1923,6 +1963,9 @@
       <c r="E2" s="13">
         <v>1</v>
       </c>
+      <c r="F2" s="13">
+        <v>0.93</v>
+      </c>
     </row>
     <row r="3" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="13">
@@ -2491,7 +2534,7 @@
       </c>
       <c r="F33" s="15">
         <f t="shared" ref="F33" si="5">SUM(F2:F32) / 100</f>
-        <v>0</v>
+        <v>9.300000000000001E-3</v>
       </c>
       <c r="G33" s="14" t="s">
         <v>10</v>

</xml_diff>